<commit_message>
refactor(data): унификация niche_id (NAIL→MANICURE, PHARMA→PHARMACY, TIRE→TIRESERVICE, WATER→WATERPLANT, CYBERCLUB→COMPCLUB)
Приводим имена per-niche xlsx к каноническим ID из config/niches.yaml.
Также обновляем niche_id значения в 14_competitors.xlsx, 15_failure_cases.xlsx
и 17_permits.xlsx (активно читаются движком). В коде engine/pdf_gen/report
словари NICHE_NAMES/NICHE_ICONS/eq_notes перепривязываются на новые ID
(полное удаление этих словарей — в шагах 6-8).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/kz/14_competitors.xlsx
+++ b/data/kz/14_competitors.xlsx
@@ -527,6 +527,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="40" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -1760,7 +1761,7 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>PHARMA</t>
+          <t>PHARMACY</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -1811,7 +1812,7 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>PHARMA</t>
+          <t>PHARMACY</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
@@ -1862,7 +1863,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>PHARMA</t>
+          <t>PHARMACY</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -1909,7 +1910,7 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>PHARMA</t>
+          <t>PHARMACY</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
@@ -2247,6 +2248,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="40" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>

</xml_diff>